<commit_message>
Update describe and gpt_example files D
</commit_message>
<xml_diff>
--- a/data/gpt_examples/team_buildup.xlsx
+++ b/data/gpt_examples/team_buildup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henri\Desktop\Fotballanalyser\context_engineering_test\Context-Engineering-TWELVE-team-work\data\gpt_examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E9CFAD-41A7-470C-BA2C-CE77E87544F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFF683A7-6CA9-4389-90AE-AFD2A52135C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,26 +69,26 @@
     <t>Optional content type label. Set to 'qa' for all rows here.</t>
   </si>
   <si>
-    <t>Here is a statistical description of Tottenhams performance in build-up, compared ot other teams.                                                               Tottenham was poor in build-ups that progress into midfield compared to other teams.Tottenham was average in build-ups that progress into a finish phase compared to other teams.Tottenham was poor in turnovers during build-up compared to other teams.Tottenham was poor in opposition box entries shortly after turnovers compared to other teams.Tottenham was poor in opposition shot probability shortly after turnovers compared to other teams.Tottenham was outstanding in build-ups that break the first defensive line of pressure compared to other teams.</t>
-  </si>
-  <si>
-    <t>Brentford FC was average in build-ups that progress into midfield compared to other teams. Brentford FC was average in build-ups that progress into a finish phase compared to other teams.Brentford FC was below average in turnovers during build-up compared to other teams.Brentford FC was good in opposition box entries shortly after turnovers compared to other teams.Brentford FC was good in opposition shot probability shortly after turnovers compared to other teams.Brentford FC was average in build-ups that break the first defensive line of pressure compared to other teams</t>
-  </si>
-  <si>
-    <t>Here is a statistical description of Manchester City's performance in build-up. The team is compared to other teams.
-Manchester City was average in build-ups that progress into midfield compared to other teams. Manchester City was outstanding for build-ups that progress into a finish phase compared to other teams in the dataset. Manchester City was good in avoiding turnovers during build-up compared to other teams in the dataset. Manchester City was average in limiting opposition box entries shortly after turnovers compared to other teams in the dataset. Manchester City was below average in limiting opposition shot probability shortly after turnovers compared to other teams in the dataset. Manchester City was good in breaking the first defensive line during build-up compared to other teams in the dataset.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manchester City is showing exceptional ability to play out from the back, and often manage to move the ball forward with control. Their skill of finding the linebreaking pass combined with extrordinary ability to get the ball from own third to attacking third is rare, and signalling a team that know how to use the pockets of space that appear in the opposition press. However, when they do loose possession in their own third, they struggle to keep opponent away from finding shooting opportunities.  Their level of getting into the middle third was mediocre, showing room for improvement against high press. Overall, Manchester City is one of the best teams in the build-up phase.  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brentford  is showing adequate level of controlling the ball while progressing the ball forward in their build-ups.  When they loose the ball, they are strong to prevent opposition from enter the box and create shooting opportunities. They are below par for turnovers, which tells they can improve their control and execution in possession. Their ability to progress into midfield and the final third are standard; they can play through a high press, but there are better teams in progressing the ball. Overall, Brentford is on a medium level when it comes to the build-up phase. </t>
-  </si>
-  <si>
-    <t>Tottenham have big room for improvement when it comes to control the ball during build-ups, and they often get into trouble when they try to play out from the back. They are exceptional at playing through the first line of pressure. However, they struggle to progress further into midfield,  and concede a lot of turnovers which often ends in shooting opportunities for the opposition. They are mediocre when is comes to get the ball into the final third. Tottenham are one of the weaker teams in the build-up phase.</t>
-  </si>
-  <si>
     <t>Example text from forward file: Giroud is a clinical forward, receiving the ball in the final third and scoring goals. His exceptional non-penalty expected goals demonstrate that it is not by chance that he has scored so many goals this season: when he gets the ball in the final third, he often finds a way to create a good chance. While he is strong in the air, he doesn’t win the ball much on the ground and he tends to score himself rather than assisting others. Giroud is one of the absolute best goal-scoring forwards in the league.</t>
+  </si>
+  <si>
+    <t>Team C have big room for improvement when it comes to control the ball during build-ups, and they often get into trouble when they try to play out from the back. They are exceptional at playing through the first line of pressure. However, they struggle to progress further into midfield,  and concede a lot of turnovers which often ends in shooting opportunities for the opposition. They are mediocre when is comes to get the ball into the final third. Team C are one of the weaker teams in the build-up phase.</t>
+  </si>
+  <si>
+    <t>Here is a statistical description of Team A's performance in build-up, compared to other teams. Team A
+was average in build-ups that progress into midfield compared to other teams. Team A was outstanding for build-ups that progress into a finish phase compared to other teams in the dataset.  Team A was good in avoiding turnovers during build-up compared to other teams in the dataset.  Team A was average in limiting opposition box entries shortly after turnovers compared to other teams in the dataset.  Team A was below average in limiting opposition shot probability shortly after turnovers compared to other teams in the dataset.  Team A was good in breaking the first defensive line during build-up compared to other teams in the dataset.</t>
+  </si>
+  <si>
+    <t>Team B was average in build-ups that progress into midfield compared to other teams. Team B was average in build-ups that progress into a finish phase compared to other teams.Team B was below average in turnovers during build-up compared to other teams.Team B was good in opposition box entries shortly after turnovers compared to other teams.Team B was good in opposition shot probability shortly after turnovers compared to other teams.Team B was average in build-ups that break the first defensive line of pressure compared to other teams</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team B  is showing adequate level of controlling the ball while progressing the ball forward in their build-ups.  When they loose the ball, they are strong to prevent opposition from enter the box and create shooting opportunities. They are below par for avoiding turnovers, which tells they can improve their control and execution in possession. Their ability to progress into midfield and the final third are standard; they can play through a high press, but there are better teams in progressing the ball. Overall, Brentford is on a medium level when it comes to the build-up phase. </t>
+  </si>
+  <si>
+    <t>Here is a statistical description of Team Cs performance in build-up, compared ot other teams.                                                                         Team C was poor in build-ups that progress into midfield compared to other teams.Team C was average in build-ups that progress into a finish phase compared to other teams.Team C was poor in turnovers during build-up compared to other teams.Team C was poor in opposition box entries shortly after turnovers compared to other teams.Team C was poor in opposition shot probability shortly after turnovers compared to other teams.Team C was outstanding in build-ups that break the first defensive line of pressure compared to other teams.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team A is showing exceptional ability to play out from the back, and often manage to move the ball forward up the pitch with control. Their are often trying to break the opposition press with linebreaking passes. Their skill of finding the linebreaking pass combined with extrordinary ability to get the ball from own third to attacking third is rare, and signalling a team that know how to use the pockets of space that appear in the opposition press. However, when they do lose possession in build-up, they struggle to stop opponent from finding shooting opportunities.  Their level of getting into the middle third was mediocre, showing room for improvement against high press. Overall, Team A is one of the best teams in the build-up phase.  </t>
   </si>
 </sst>
 </file>
@@ -502,19 +502,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="174" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>14</v>
@@ -524,13 +524,13 @@
     </row>
     <row r="4" spans="1:4" ht="159.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="D4" s="2"/>
     </row>
@@ -770,8 +770,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>